<commit_message>
taxdome migration import endpoints and settings tab
</commit_message>
<xml_diff>
--- a/JAMM_PX_Master_Build_Schedule.xlsx
+++ b/JAMM_PX_Master_Build_Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andre\Downloads\JAMM-Media\JAMM OS Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97B8BF64-52A9-426C-832B-F87137964A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7D9D48-2A91-4257-AE27-4A15D5691334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="420">
   <si>
     <t>JAMM PX — Master Build Schedule  |  Now → August 15, 2026  |  Chronological — both owners interleaved</t>
   </si>
@@ -1276,6 +1276,12 @@
   </si>
   <si>
     <t>Production environment audit complete</t>
+  </si>
+  <si>
+    <t>✅ Complete</t>
+  </si>
+  <si>
+    <t>🟡 Waiting</t>
   </si>
 </sst>
 </file>
@@ -1613,14 +1619,14 @@
     <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2050,7 +2056,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="35" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="33"/>
@@ -2087,7 +2093,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>12</v>
@@ -2104,7 +2110,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>14</v>
@@ -2121,7 +2127,7 @@
         <v>0.25</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>16</v>
@@ -2138,7 +2144,7 @@
         <v>0.25</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>18</v>
@@ -2164,7 +2170,7 @@
         <v>2</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>21</v>
@@ -2181,7 +2187,7 @@
         <v>2</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>11</v>
+        <v>419</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>23</v>
@@ -2198,7 +2204,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>25</v>
@@ -2215,7 +2221,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>27</v>
@@ -2232,7 +2238,7 @@
         <v>0.5</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>29</v>
@@ -2249,7 +2255,7 @@
         <v>1</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E16" s="9"/>
     </row>
@@ -2280,7 +2286,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A19" s="32" t="s">
+      <c r="A19" s="35" t="s">
         <v>36</v>
       </c>
       <c r="B19" s="33"/>
@@ -2317,7 +2323,7 @@
         <v>2</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>40</v>
@@ -2334,7 +2340,7 @@
         <v>2</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E23" s="9"/>
     </row>
@@ -2349,7 +2355,7 @@
         <v>0.5</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>43</v>
@@ -2366,7 +2372,7 @@
         <v>1</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>45</v>
@@ -2426,7 +2432,7 @@
         <v>1</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E29" s="14" t="s">
         <v>52</v>
@@ -2482,7 +2488,7 @@
       <c r="E32" s="17"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A33" s="32" t="s">
+      <c r="A33" s="35" t="s">
         <v>58</v>
       </c>
       <c r="B33" s="33"/>
@@ -2519,7 +2525,7 @@
         <v>3</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>62</v>
@@ -2536,7 +2542,7 @@
         <v>2</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>64</v>
@@ -2553,7 +2559,7 @@
         <v>3</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E38" s="6"/>
     </row>
@@ -2568,7 +2574,7 @@
         <v>1</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E39" s="9"/>
     </row>
@@ -2583,7 +2589,7 @@
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E40" s="6"/>
     </row>
@@ -2675,7 +2681,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E46" s="14"/>
     </row>
@@ -2690,7 +2696,7 @@
         <v>1</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E47" s="17"/>
     </row>
@@ -2705,7 +2711,7 @@
         <v>0.5</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E48" s="14"/>
     </row>
@@ -2750,7 +2756,7 @@
         <v>1</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E51" s="17" t="s">
         <v>82</v>
@@ -2804,7 +2810,7 @@
       <c r="E54" s="14"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A55" s="32" t="s">
+      <c r="A55" s="35" t="s">
         <v>87</v>
       </c>
       <c r="B55" s="33"/>
@@ -2841,7 +2847,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E58" s="6"/>
     </row>
@@ -2856,7 +2862,7 @@
         <v>2</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E59" s="9"/>
     </row>
@@ -2871,7 +2877,7 @@
         <v>5</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>11</v>
+        <v>419</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>93</v>
@@ -2953,7 +2959,7 @@
       </c>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A66" s="32" t="s">
+      <c r="A66" s="35" t="s">
         <v>102</v>
       </c>
       <c r="B66" s="33"/>
@@ -3050,7 +3056,7 @@
         <v>1</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E73" s="14" t="s">
         <v>113</v>
@@ -3155,7 +3161,7 @@
       </c>
     </row>
     <row r="80" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A80" s="32" t="s">
+      <c r="A80" s="35" t="s">
         <v>124</v>
       </c>
       <c r="B80" s="33"/>
@@ -3441,7 +3447,7 @@
       </c>
     </row>
     <row r="100" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A100" s="32" t="s">
+      <c r="A100" s="35" t="s">
         <v>148</v>
       </c>
       <c r="B100" s="33"/>
@@ -3647,7 +3653,7 @@
       </c>
     </row>
     <row r="114" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A114" s="32" t="s">
+      <c r="A114" s="35" t="s">
         <v>173</v>
       </c>
       <c r="B114" s="33"/>
@@ -3881,7 +3887,7 @@
       </c>
     </row>
     <row r="130" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A130" s="32" t="s">
+      <c r="A130" s="35" t="s">
         <v>198</v>
       </c>
       <c r="B130" s="33"/>
@@ -4087,7 +4093,7 @@
       </c>
     </row>
     <row r="144" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A144" s="32" t="s">
+      <c r="A144" s="35" t="s">
         <v>222</v>
       </c>
       <c r="B144" s="33"/>
@@ -4232,7 +4238,7 @@
       <c r="E154" s="14"/>
     </row>
     <row r="155" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A155" s="32" t="s">
+      <c r="A155" s="35" t="s">
         <v>235</v>
       </c>
       <c r="B155" s="33"/>
@@ -4250,7 +4256,7 @@
       <c r="E156" s="33"/>
     </row>
     <row r="157" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A157" s="35" t="s">
+      <c r="A157" s="32" t="s">
         <v>237</v>
       </c>
       <c r="B157" s="33"/>
@@ -4308,7 +4314,7 @@
       <c r="E160" s="22"/>
     </row>
     <row r="161" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A161" s="35" t="s">
+      <c r="A161" s="32" t="s">
         <v>244</v>
       </c>
       <c r="B161" s="33"/>
@@ -4435,7 +4441,7 @@
       </c>
     </row>
     <row r="170" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A170" s="32" t="s">
+      <c r="A170" s="35" t="s">
         <v>255</v>
       </c>
       <c r="B170" s="33"/>
@@ -4469,30 +4475,10 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="A161:E161"/>
-    <mergeCell ref="A171:E171"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A170:E170"/>
-    <mergeCell ref="A102:E102"/>
-    <mergeCell ref="A115:E115"/>
-    <mergeCell ref="A155:E155"/>
-    <mergeCell ref="A167:E167"/>
-    <mergeCell ref="A67:E67"/>
-    <mergeCell ref="A130:E130"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A100:E100"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A81:E81"/>
-    <mergeCell ref="A96:E96"/>
-    <mergeCell ref="A72:E72"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A116:E116"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A126:E126"/>
-    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A149:E149"/>
+    <mergeCell ref="A144:E144"/>
+    <mergeCell ref="A131:E131"/>
+    <mergeCell ref="A156:E156"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A132:E132"/>
     <mergeCell ref="A61:E61"/>
@@ -4509,15 +4495,35 @@
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A100:E100"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A161:E161"/>
+    <mergeCell ref="A171:E171"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A170:E170"/>
+    <mergeCell ref="A102:E102"/>
+    <mergeCell ref="A115:E115"/>
+    <mergeCell ref="A155:E155"/>
+    <mergeCell ref="A167:E167"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A130:E130"/>
+    <mergeCell ref="A116:E116"/>
+    <mergeCell ref="A126:E126"/>
     <mergeCell ref="A114:E114"/>
-    <mergeCell ref="A34:E34"/>
     <mergeCell ref="A157:E157"/>
-    <mergeCell ref="A82:E82"/>
     <mergeCell ref="A138:E138"/>
-    <mergeCell ref="A149:E149"/>
-    <mergeCell ref="A144:E144"/>
-    <mergeCell ref="A131:E131"/>
-    <mergeCell ref="A156:E156"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:E173">
     <cfRule type="expression" dxfId="5" priority="1">

</xml_diff>

<commit_message>
email calendar integration session 1 - per-staff OAuth architecture
</commit_message>
<xml_diff>
--- a/JAMM_PX_Master_Build_Schedule.xlsx
+++ b/JAMM_PX_Master_Build_Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andre\Downloads\JAMM-Media\JAMM OS Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7D9D48-2A91-4257-AE27-4A15D5691334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F00A536-BA8F-45E5-A162-24500735364E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1619,20 +1619,20 @@
     <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2056,7 +2056,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="37" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="33"/>
@@ -2065,7 +2065,7 @@
       <c r="E3" s="33"/>
     </row>
     <row r="4" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="36" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="33"/>
@@ -2074,7 +2074,7 @@
       <c r="E4" s="33"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="34" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="33"/>
@@ -2151,7 +2151,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="34" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="33"/>
@@ -2260,7 +2260,7 @@
       <c r="E16" s="9"/>
     </row>
     <row r="17" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A17" s="37" t="s">
+      <c r="A17" s="32" t="s">
         <v>31</v>
       </c>
       <c r="B17" s="33"/>
@@ -2286,7 +2286,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A19" s="35" t="s">
+      <c r="A19" s="37" t="s">
         <v>36</v>
       </c>
       <c r="B19" s="33"/>
@@ -2295,7 +2295,7 @@
       <c r="E19" s="33"/>
     </row>
     <row r="20" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A20" s="34" t="s">
+      <c r="A20" s="36" t="s">
         <v>37</v>
       </c>
       <c r="B20" s="33"/>
@@ -2304,7 +2304,7 @@
       <c r="E20" s="33"/>
     </row>
     <row r="21" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="34" t="s">
         <v>38</v>
       </c>
       <c r="B21" s="33"/>
@@ -2379,7 +2379,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A26" s="37" t="s">
+      <c r="A26" s="32" t="s">
         <v>46</v>
       </c>
       <c r="B26" s="33"/>
@@ -2415,7 +2415,7 @@
         <v>3</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E28" s="17" t="s">
         <v>50</v>
@@ -2449,7 +2449,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E30" s="17" t="s">
         <v>54</v>
@@ -2488,7 +2488,7 @@
       <c r="E32" s="17"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A33" s="35" t="s">
+      <c r="A33" s="37" t="s">
         <v>58</v>
       </c>
       <c r="B33" s="33"/>
@@ -2497,7 +2497,7 @@
       <c r="E33" s="33"/>
     </row>
     <row r="34" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A34" s="34" t="s">
+      <c r="A34" s="36" t="s">
         <v>59</v>
       </c>
       <c r="B34" s="33"/>
@@ -2506,7 +2506,7 @@
       <c r="E34" s="33"/>
     </row>
     <row r="35" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A35" s="36" t="s">
+      <c r="A35" s="34" t="s">
         <v>60</v>
       </c>
       <c r="B35" s="33"/>
@@ -2594,7 +2594,7 @@
       <c r="E40" s="6"/>
     </row>
     <row r="41" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A41" s="37" t="s">
+      <c r="A41" s="32" t="s">
         <v>68</v>
       </c>
       <c r="B41" s="33"/>
@@ -2613,7 +2613,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E42" s="14" t="s">
         <v>70</v>
@@ -2630,7 +2630,7 @@
         <v>2</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E43" s="17" t="s">
         <v>72</v>
@@ -2647,7 +2647,7 @@
         <v>2</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>72</v>
@@ -2726,7 +2726,7 @@
         <v>0.5</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E49" s="17"/>
     </row>
@@ -2741,7 +2741,7 @@
         <v>1</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E50" s="14"/>
     </row>
@@ -2773,7 +2773,7 @@
         <v>0.5</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E52" s="14" t="s">
         <v>84</v>
@@ -2810,7 +2810,7 @@
       <c r="E54" s="14"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A55" s="35" t="s">
+      <c r="A55" s="37" t="s">
         <v>87</v>
       </c>
       <c r="B55" s="33"/>
@@ -2819,7 +2819,7 @@
       <c r="E55" s="33"/>
     </row>
     <row r="56" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A56" s="34" t="s">
+      <c r="A56" s="36" t="s">
         <v>88</v>
       </c>
       <c r="B56" s="33"/>
@@ -2828,7 +2828,7 @@
       <c r="E56" s="33"/>
     </row>
     <row r="57" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A57" s="36" t="s">
+      <c r="A57" s="34" t="s">
         <v>89</v>
       </c>
       <c r="B57" s="33"/>
@@ -2884,7 +2884,7 @@
       </c>
     </row>
     <row r="61" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A61" s="37" t="s">
+      <c r="A61" s="32" t="s">
         <v>94</v>
       </c>
       <c r="B61" s="33"/>
@@ -2959,7 +2959,7 @@
       </c>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A66" s="35" t="s">
+      <c r="A66" s="37" t="s">
         <v>102</v>
       </c>
       <c r="B66" s="33"/>
@@ -2968,7 +2968,7 @@
       <c r="E66" s="33"/>
     </row>
     <row r="67" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A67" s="34" t="s">
+      <c r="A67" s="36" t="s">
         <v>103</v>
       </c>
       <c r="B67" s="33"/>
@@ -2977,7 +2977,7 @@
       <c r="E67" s="33"/>
     </row>
     <row r="68" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A68" s="36" t="s">
+      <c r="A68" s="34" t="s">
         <v>104</v>
       </c>
       <c r="B68" s="33"/>
@@ -3037,7 +3037,7 @@
       </c>
     </row>
     <row r="72" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A72" s="37" t="s">
+      <c r="A72" s="32" t="s">
         <v>111</v>
       </c>
       <c r="B72" s="33"/>
@@ -3090,7 +3090,7 @@
         <v>1.5</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E75" s="14"/>
     </row>
@@ -3105,7 +3105,7 @@
         <v>1.5</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="E76" s="17"/>
     </row>
@@ -3161,7 +3161,7 @@
       </c>
     </row>
     <row r="80" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A80" s="35" t="s">
+      <c r="A80" s="37" t="s">
         <v>124</v>
       </c>
       <c r="B80" s="33"/>
@@ -3170,7 +3170,7 @@
       <c r="E80" s="33"/>
     </row>
     <row r="81" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A81" s="34" t="s">
+      <c r="A81" s="36" t="s">
         <v>125</v>
       </c>
       <c r="B81" s="33"/>
@@ -3179,7 +3179,7 @@
       <c r="E81" s="33"/>
     </row>
     <row r="82" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A82" s="36" t="s">
+      <c r="A82" s="34" t="s">
         <v>126</v>
       </c>
       <c r="B82" s="33"/>
@@ -3389,7 +3389,7 @@
       </c>
     </row>
     <row r="96" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A96" s="37" t="s">
+      <c r="A96" s="32" t="s">
         <v>143</v>
       </c>
       <c r="B96" s="33"/>
@@ -3447,7 +3447,7 @@
       </c>
     </row>
     <row r="100" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A100" s="35" t="s">
+      <c r="A100" s="37" t="s">
         <v>148</v>
       </c>
       <c r="B100" s="33"/>
@@ -3456,7 +3456,7 @@
       <c r="E100" s="33"/>
     </row>
     <row r="101" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A101" s="34" t="s">
+      <c r="A101" s="36" t="s">
         <v>149</v>
       </c>
       <c r="B101" s="33"/>
@@ -3465,7 +3465,7 @@
       <c r="E101" s="33"/>
     </row>
     <row r="102" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A102" s="36" t="s">
+      <c r="A102" s="34" t="s">
         <v>150</v>
       </c>
       <c r="B102" s="33"/>
@@ -3559,7 +3559,7 @@
       </c>
     </row>
     <row r="108" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A108" s="37" t="s">
+      <c r="A108" s="32" t="s">
         <v>162</v>
       </c>
       <c r="B108" s="33"/>
@@ -3653,7 +3653,7 @@
       </c>
     </row>
     <row r="114" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A114" s="35" t="s">
+      <c r="A114" s="37" t="s">
         <v>173</v>
       </c>
       <c r="B114" s="33"/>
@@ -3662,7 +3662,7 @@
       <c r="E114" s="33"/>
     </row>
     <row r="115" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A115" s="34" t="s">
+      <c r="A115" s="36" t="s">
         <v>174</v>
       </c>
       <c r="B115" s="33"/>
@@ -3671,7 +3671,7 @@
       <c r="E115" s="33"/>
     </row>
     <row r="116" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A116" s="36" t="s">
+      <c r="A116" s="34" t="s">
         <v>175</v>
       </c>
       <c r="B116" s="33"/>
@@ -3827,7 +3827,7 @@
       <c r="E125" s="6"/>
     </row>
     <row r="126" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A126" s="37" t="s">
+      <c r="A126" s="32" t="s">
         <v>191</v>
       </c>
       <c r="B126" s="33"/>
@@ -3887,7 +3887,7 @@
       </c>
     </row>
     <row r="130" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A130" s="35" t="s">
+      <c r="A130" s="37" t="s">
         <v>198</v>
       </c>
       <c r="B130" s="33"/>
@@ -3896,7 +3896,7 @@
       <c r="E130" s="33"/>
     </row>
     <row r="131" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A131" s="34" t="s">
+      <c r="A131" s="36" t="s">
         <v>199</v>
       </c>
       <c r="B131" s="33"/>
@@ -3905,7 +3905,7 @@
       <c r="E131" s="33"/>
     </row>
     <row r="132" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A132" s="36" t="s">
+      <c r="A132" s="34" t="s">
         <v>200</v>
       </c>
       <c r="B132" s="33"/>
@@ -3999,7 +3999,7 @@
       </c>
     </row>
     <row r="138" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A138" s="37" t="s">
+      <c r="A138" s="32" t="s">
         <v>211</v>
       </c>
       <c r="B138" s="33"/>
@@ -4093,7 +4093,7 @@
       </c>
     </row>
     <row r="144" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A144" s="35" t="s">
+      <c r="A144" s="37" t="s">
         <v>222</v>
       </c>
       <c r="B144" s="33"/>
@@ -4102,7 +4102,7 @@
       <c r="E144" s="33"/>
     </row>
     <row r="145" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A145" s="34" t="s">
+      <c r="A145" s="36" t="s">
         <v>223</v>
       </c>
       <c r="B145" s="33"/>
@@ -4111,7 +4111,7 @@
       <c r="E145" s="33"/>
     </row>
     <row r="146" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A146" s="36" t="s">
+      <c r="A146" s="34" t="s">
         <v>224</v>
       </c>
       <c r="B146" s="33"/>
@@ -4150,7 +4150,7 @@
       <c r="E148" s="9"/>
     </row>
     <row r="149" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A149" s="37" t="s">
+      <c r="A149" s="32" t="s">
         <v>227</v>
       </c>
       <c r="B149" s="33"/>
@@ -4238,7 +4238,7 @@
       <c r="E154" s="14"/>
     </row>
     <row r="155" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A155" s="35" t="s">
+      <c r="A155" s="37" t="s">
         <v>235</v>
       </c>
       <c r="B155" s="33"/>
@@ -4247,7 +4247,7 @@
       <c r="E155" s="33"/>
     </row>
     <row r="156" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A156" s="34" t="s">
+      <c r="A156" s="36" t="s">
         <v>236</v>
       </c>
       <c r="B156" s="33"/>
@@ -4256,7 +4256,7 @@
       <c r="E156" s="33"/>
     </row>
     <row r="157" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A157" s="32" t="s">
+      <c r="A157" s="35" t="s">
         <v>237</v>
       </c>
       <c r="B157" s="33"/>
@@ -4314,7 +4314,7 @@
       <c r="E160" s="22"/>
     </row>
     <row r="161" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A161" s="32" t="s">
+      <c r="A161" s="35" t="s">
         <v>244</v>
       </c>
       <c r="B161" s="33"/>
@@ -4400,7 +4400,7 @@
       <c r="E166" s="22"/>
     </row>
     <row r="167" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A167" s="37" t="s">
+      <c r="A167" s="32" t="s">
         <v>251</v>
       </c>
       <c r="B167" s="33"/>
@@ -4441,7 +4441,7 @@
       </c>
     </row>
     <row r="170" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A170" s="35" t="s">
+      <c r="A170" s="37" t="s">
         <v>255</v>
       </c>
       <c r="B170" s="33"/>
@@ -4450,7 +4450,7 @@
       <c r="E170" s="33"/>
     </row>
     <row r="171" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A171" s="34" t="s">
+      <c r="A171" s="36" t="s">
         <v>256</v>
       </c>
       <c r="B171" s="33"/>
@@ -4475,10 +4475,6 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="A149:E149"/>
-    <mergeCell ref="A144:E144"/>
-    <mergeCell ref="A131:E131"/>
-    <mergeCell ref="A156:E156"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A132:E132"/>
     <mergeCell ref="A61:E61"/>
@@ -4491,10 +4487,6 @@
     <mergeCell ref="A145:E145"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A57:E57"/>
-    <mergeCell ref="A101:E101"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A100:E100"/>
     <mergeCell ref="A20:E20"/>
@@ -4507,6 +4499,16 @@
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A157:E157"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A149:E149"/>
+    <mergeCell ref="A144:E144"/>
+    <mergeCell ref="A131:E131"/>
+    <mergeCell ref="A156:E156"/>
+    <mergeCell ref="A138:E138"/>
     <mergeCell ref="A82:E82"/>
     <mergeCell ref="A161:E161"/>
     <mergeCell ref="A171:E171"/>
@@ -4522,8 +4524,6 @@
     <mergeCell ref="A116:E116"/>
     <mergeCell ref="A126:E126"/>
     <mergeCell ref="A114:E114"/>
-    <mergeCell ref="A157:E157"/>
-    <mergeCell ref="A138:E138"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:E173">
     <cfRule type="expression" dxfId="5" priority="1">

</xml_diff>